<commit_message>
update test case file
</commit_message>
<xml_diff>
--- a/GSA SQA_Test_Cases.xlsx
+++ b/GSA SQA_Test_Cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -92,12 +92,6 @@
     <t>TC-06</t>
   </si>
   <si>
-    <t>Create assignment with empty fields</t>
-  </si>
-  <si>
-    <t>Submit without filling fields</t>
-  </si>
-  <si>
     <t>Validation error</t>
   </si>
   <si>
@@ -249,9 +243,6 @@
   </si>
   <si>
     <t>Redirect to login</t>
-  </si>
-  <si>
-    <t>TC-20</t>
   </si>
   <si>
     <t>API access without JWT</t>
@@ -666,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -683,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
         <v>82</v>
-      </c>
-      <c r="C1" t="s">
-        <v>85</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -701,7 +692,7 @@
         <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -709,7 +700,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -724,7 +715,7 @@
         <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -732,7 +723,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -747,7 +738,7 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -755,7 +746,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -770,7 +761,7 @@
         <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -778,7 +769,7 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
@@ -793,7 +784,7 @@
         <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -801,7 +792,7 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
@@ -816,7 +807,7 @@
         <v>23</v>
       </c>
       <c r="G6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -824,254 +815,246 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="G8" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" t="s">
         <v>37</v>
       </c>
-      <c r="D10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" t="s">
-        <v>39</v>
-      </c>
       <c r="G10" t="s">
-        <v>86</v>
+        <v>101</v>
+      </c>
+      <c r="H10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
-      </c>
-      <c r="H11" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
         <v>78</v>
-      </c>
-      <c r="C21" t="s">
-        <v>79</v>
-      </c>
-      <c r="D21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1098,16 +1081,16 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" t="s">
         <v>87</v>
-      </c>
-      <c r="B1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" t="s">
-        <v>90</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -1116,48 +1099,48 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I1" t="s">
         <v>4</v>
       </c>
       <c r="J1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" t="s">
         <v>94</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>95</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>96</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>97</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>98</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>99</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>100</v>
-      </c>
-      <c r="H2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I2" t="s">
-        <v>102</v>
-      </c>
-      <c r="J2" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>